<commit_message>
excel import page implemented
</commit_message>
<xml_diff>
--- a/src/assets/urun_liste_demo.xlsx
+++ b/src/assets/urun_liste_demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ismai\Desktop\Kodlar\turkcell\trkcell-reat\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D5966D3-4671-4FDC-BCB2-DEC7AB93934D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{504FF5D4-1EC0-49E0-A0CF-6B0C1D29CD64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A916BB5B-F7EE-4D93-8B39-99FF5397B351}"/>
   </bookViews>
@@ -38,40 +38,40 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
+    <t>Kalem pil</t>
+  </si>
+  <si>
+    <t>Kırtasiye</t>
+  </si>
+  <si>
+    <t>Duracell</t>
+  </si>
+  <si>
+    <t>AA 4lü</t>
+  </si>
+  <si>
+    <t>Adet</t>
+  </si>
+  <si>
+    <t>Soda</t>
+  </si>
+  <si>
+    <t>Mutfak</t>
+  </si>
+  <si>
+    <t>Beypazarı</t>
+  </si>
+  <si>
+    <t>Cam Şişe</t>
+  </si>
+  <si>
+    <t>Birim</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
     <t>Marka</t>
-  </si>
-  <si>
-    <t>Model</t>
-  </si>
-  <si>
-    <t>Birim</t>
-  </si>
-  <si>
-    <t>Kalem pil</t>
-  </si>
-  <si>
-    <t>Kırtasiye</t>
-  </si>
-  <si>
-    <t>Duracell</t>
-  </si>
-  <si>
-    <t>AA 4lü</t>
-  </si>
-  <si>
-    <t>Adet</t>
-  </si>
-  <si>
-    <t>Soda</t>
-  </si>
-  <si>
-    <t>Mutfak</t>
-  </si>
-  <si>
-    <t>Beypazarı</t>
-  </si>
-  <si>
-    <t>Cam Şişe</t>
   </si>
   <si>
     <t>Ürün grubu</t>
@@ -538,7 +538,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" customWidth="1"/>
     <col min="3" max="3" width="13.44140625" customWidth="1"/>
     <col min="4" max="4" width="16.44140625" customWidth="1"/>
     <col min="5" max="5" width="12.44140625" customWidth="1"/>
@@ -552,47 +552,47 @@
         <v>12</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>4</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>